<commit_message>
Synchronisation de mon application vers Google sheets OK
</commit_message>
<xml_diff>
--- a/docs/Modele-Agenda-GestionAgenda.xlsx
+++ b/docs/Modele-Agenda-GestionAgenda.xlsx
@@ -125,7 +125,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="10">
     <dxf>
       <font>
         <strike val="1"/>
@@ -168,6 +168,13 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFEDD5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00DBEAFE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -54727,16 +54734,19 @@
       <formula>$O2="Reporté"</formula>
     </cfRule>
     <cfRule type="expression" priority="6" dxfId="5" stopIfTrue="1">
+      <formula>$O2="Accepté"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="6" stopIfTrue="1">
       <formula>OR($G2="Déplacement",$G2="Temps bloqué",$G2="Personnel",$G2="Événement")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2:N2001">
-    <cfRule type="expression" priority="7" dxfId="6">
+    <cfRule type="expression" priority="8" dxfId="7">
       <formula>OR($N2="Haute",$N2="Critique")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q2:Q2001">
-    <cfRule type="expression" priority="8" dxfId="7">
+    <cfRule type="expression" priority="9" dxfId="8">
       <formula>AND($Q2="Non",$B2&lt;&gt;"",$B2-TODAY()&lt;=1,$B2&gt;=TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
@@ -54748,7 +54758,7 @@
       <formula1>=Listes!$B$2:$B$5</formula1>
     </dataValidation>
     <dataValidation sqref="O2:O2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Choisissez un statut de la liste." type="list">
-      <formula1>=Listes!$C$2:$C$7</formula1>
+      <formula1>=Listes!$C$2:$C$8</formula1>
     </dataValidation>
     <dataValidation sqref="Q2:Q2001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valeur non reconnue" error="Oui ou Non." type="list">
       <formula1>=Listes!$D$2:$D$3</formula1>
@@ -57317,10 +57327,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:F501">
-    <cfRule type="expression" priority="1" dxfId="6">
+    <cfRule type="expression" priority="1" dxfId="7">
       <formula>AND($E2&lt;&gt;"",$E2&lt;TODAY(),$F2&lt;&gt;"Oui")</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="8">
+    <cfRule type="expression" priority="2" dxfId="9">
       <formula>$F2="Oui"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -57405,7 +57415,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Confirmé</t>
+          <t>Accepté</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -57427,7 +57437,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Reporté</t>
+          <t>Confirmé</t>
         </is>
       </c>
     </row>
@@ -57444,7 +57454,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Refusé</t>
+          <t>Reporté</t>
         </is>
       </c>
     </row>
@@ -57456,7 +57466,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Annulé</t>
+          <t>Refusé</t>
         </is>
       </c>
     </row>
@@ -57468,7 +57478,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>Annulé</t>
         </is>
       </c>
     </row>
@@ -57476,6 +57486,11 @@
       <c r="A8" t="inlineStr">
         <is>
           <t>Événement</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Terminé</t>
         </is>
       </c>
     </row>

</xml_diff>